<commit_message>
New updated all class scraper
</commit_message>
<xml_diff>
--- a/CFTR2_25September2024.xlsx
+++ b/CFTR2_25September2024.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\adith\Documents\Cystic Fibrosis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/24C5ABD427167479/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04C04561-E51B-4E11-AB4A-4473DBB0F973}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="534" documentId="8_{9CA877D2-2B71-403A-8B7B-C14BB5CCBE55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{45A6C097-862F-4B72-9891-BF76B9A8DB84}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" tabRatio="822" activeTab="3" xr2:uid="{8F569A10-4B41-497D-8A1A-607ADB2C4296}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" tabRatio="822" activeTab="5" xr2:uid="{8F569A10-4B41-497D-8A1A-607ADB2C4296}"/>
   </bookViews>
   <sheets>
     <sheet name="Get Started with Python (2)" sheetId="42" r:id="rId1"/>
@@ -165,7 +165,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16774" uniqueCount="6294">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16770" uniqueCount="6294">
   <si>
     <t>9T</t>
   </si>
@@ -19799,9 +19799,6 @@
     <xf numFmtId="0" fontId="23" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -19849,6 +19846,9 @@
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -20131,6 +20131,10 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
@@ -20842,15 +20846,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="23.25">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="48" t="s">
         <v>6269</v>
       </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="49"/>
-      <c r="F1" s="49"/>
-      <c r="G1" s="49"/>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
     </row>
     <row r="3" spans="1:10" ht="23.25">
       <c r="A3" s="15" t="s">
@@ -20858,10 +20862,10 @@
       </c>
       <c r="B3" s="14"/>
       <c r="C3" s="10"/>
-      <c r="G3" s="51" t="s">
+      <c r="G3" s="50" t="s">
         <v>6267</v>
       </c>
-      <c r="H3" s="51"/>
+      <c r="H3" s="50"/>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
@@ -20908,17 +20912,17 @@
       <c r="E5" t="s">
         <v>6247</v>
       </c>
-      <c r="G5" s="48" t="s">
+      <c r="G5" s="47" t="s">
         <v>6257</v>
       </c>
-      <c r="H5" s="41" t="e" cm="1" vm="1">
+      <c r="H5" s="40" t="e" cm="1" vm="1">
         <f t="array" ref="H5">_xlfn._xlws.PY(0,1,IrisDataSet4[#All])</f>
         <v>#VALUE!</v>
       </c>
-      <c r="I5" s="42" t="s">
+      <c r="I5" s="41" t="s">
         <v>6256</v>
       </c>
-      <c r="J5" s="40"/>
+      <c r="J5" s="39"/>
     </row>
     <row r="6" spans="1:10">
       <c r="A6">
@@ -20936,10 +20940,10 @@
       <c r="E6" t="s">
         <v>6247</v>
       </c>
-      <c r="G6" s="48"/>
-      <c r="H6" s="41"/>
-      <c r="I6" s="42"/>
-      <c r="J6" s="40"/>
+      <c r="G6" s="47"/>
+      <c r="H6" s="40"/>
+      <c r="I6" s="41"/>
+      <c r="J6" s="39"/>
     </row>
     <row r="7" spans="1:10">
       <c r="A7">
@@ -20957,10 +20961,10 @@
       <c r="E7" t="s">
         <v>6247</v>
       </c>
-      <c r="G7" s="48"/>
-      <c r="H7" s="41"/>
-      <c r="I7" s="42"/>
-      <c r="J7" s="40"/>
+      <c r="G7" s="47"/>
+      <c r="H7" s="40"/>
+      <c r="I7" s="41"/>
+      <c r="J7" s="39"/>
     </row>
     <row r="8" spans="1:10">
       <c r="A8">
@@ -20978,10 +20982,10 @@
       <c r="E8" t="s">
         <v>6247</v>
       </c>
-      <c r="G8" s="48"/>
-      <c r="H8" s="41"/>
-      <c r="I8" s="42"/>
-      <c r="J8" s="40"/>
+      <c r="G8" s="47"/>
+      <c r="H8" s="40"/>
+      <c r="I8" s="41"/>
+      <c r="J8" s="39"/>
     </row>
     <row r="9" spans="1:10">
       <c r="A9">
@@ -20999,17 +21003,17 @@
       <c r="E9" t="s">
         <v>6247</v>
       </c>
-      <c r="G9" s="47" t="s">
+      <c r="G9" s="46" t="s">
         <v>6255</v>
       </c>
-      <c r="H9" s="41" t="e" cm="1" vm="2">
+      <c r="H9" s="40" t="e" cm="1" vm="2">
         <f t="array" ref="H9">_xlfn._xlws.PY(1,1)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="I9" s="42" t="s">
+      <c r="I9" s="41" t="s">
         <v>6254</v>
       </c>
-      <c r="J9" s="40"/>
+      <c r="J9" s="39"/>
     </row>
     <row r="10" spans="1:10">
       <c r="A10">
@@ -21027,10 +21031,10 @@
       <c r="E10" t="s">
         <v>6247</v>
       </c>
-      <c r="G10" s="48"/>
-      <c r="H10" s="41"/>
-      <c r="I10" s="42"/>
-      <c r="J10" s="40"/>
+      <c r="G10" s="47"/>
+      <c r="H10" s="40"/>
+      <c r="I10" s="41"/>
+      <c r="J10" s="39"/>
     </row>
     <row r="11" spans="1:10">
       <c r="A11">
@@ -21048,10 +21052,10 @@
       <c r="E11" t="s">
         <v>6247</v>
       </c>
-      <c r="G11" s="48"/>
-      <c r="H11" s="41"/>
-      <c r="I11" s="42"/>
-      <c r="J11" s="40"/>
+      <c r="G11" s="47"/>
+      <c r="H11" s="40"/>
+      <c r="I11" s="41"/>
+      <c r="J11" s="39"/>
     </row>
     <row r="12" spans="1:10">
       <c r="A12">
@@ -21069,10 +21073,10 @@
       <c r="E12" t="s">
         <v>6247</v>
       </c>
-      <c r="G12" s="48"/>
-      <c r="H12" s="41"/>
-      <c r="I12" s="42"/>
-      <c r="J12" s="40"/>
+      <c r="G12" s="47"/>
+      <c r="H12" s="40"/>
+      <c r="I12" s="41"/>
+      <c r="J12" s="39"/>
     </row>
     <row r="13" spans="1:10">
       <c r="A13">
@@ -21090,17 +21094,17 @@
       <c r="E13" t="s">
         <v>6247</v>
       </c>
-      <c r="G13" s="47" t="s">
+      <c r="G13" s="46" t="s">
         <v>6253</v>
       </c>
-      <c r="H13" s="41" t="e" cm="1" vm="3">
+      <c r="H13" s="40" t="e" cm="1" vm="3">
         <f t="array" ref="H13">_xlfn._xlws.PY(2,1)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="I13" s="42" t="s">
+      <c r="I13" s="41" t="s">
         <v>6252</v>
       </c>
-      <c r="J13" s="46"/>
+      <c r="J13" s="45"/>
     </row>
     <row r="14" spans="1:10">
       <c r="A14">
@@ -21118,10 +21122,10 @@
       <c r="E14" t="s">
         <v>6247</v>
       </c>
-      <c r="G14" s="48"/>
-      <c r="H14" s="41"/>
-      <c r="I14" s="42"/>
-      <c r="J14" s="46"/>
+      <c r="G14" s="47"/>
+      <c r="H14" s="40"/>
+      <c r="I14" s="41"/>
+      <c r="J14" s="45"/>
     </row>
     <row r="15" spans="1:10">
       <c r="A15">
@@ -21139,10 +21143,10 @@
       <c r="E15" t="s">
         <v>6247</v>
       </c>
-      <c r="G15" s="48"/>
-      <c r="H15" s="41"/>
-      <c r="I15" s="42"/>
-      <c r="J15" s="46"/>
+      <c r="G15" s="47"/>
+      <c r="H15" s="40"/>
+      <c r="I15" s="41"/>
+      <c r="J15" s="45"/>
     </row>
     <row r="16" spans="1:10">
       <c r="A16">
@@ -21160,10 +21164,10 @@
       <c r="E16" t="s">
         <v>6247</v>
       </c>
-      <c r="G16" s="48"/>
-      <c r="H16" s="41"/>
-      <c r="I16" s="42"/>
-      <c r="J16" s="46"/>
+      <c r="G16" s="47"/>
+      <c r="H16" s="40"/>
+      <c r="I16" s="41"/>
+      <c r="J16" s="45"/>
     </row>
     <row r="17" spans="1:10">
       <c r="A17">
@@ -21181,10 +21185,10 @@
       <c r="E17" t="s">
         <v>6247</v>
       </c>
-      <c r="G17" s="48"/>
-      <c r="H17" s="41"/>
-      <c r="I17" s="42"/>
-      <c r="J17" s="46"/>
+      <c r="G17" s="47"/>
+      <c r="H17" s="40"/>
+      <c r="I17" s="41"/>
+      <c r="J17" s="45"/>
     </row>
     <row r="18" spans="1:10">
       <c r="A18">
@@ -21202,17 +21206,17 @@
       <c r="E18" t="s">
         <v>6247</v>
       </c>
-      <c r="G18" s="47" t="s">
+      <c r="G18" s="46" t="s">
         <v>6251</v>
       </c>
-      <c r="H18" s="48" t="e" cm="1" vm="4">
+      <c r="H18" s="47" t="e" cm="1" vm="4">
         <f t="array" ref="H18">_xlfn._xlws.PY(3,0)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="I18" s="42" t="s">
+      <c r="I18" s="41" t="s">
         <v>6250</v>
       </c>
-      <c r="J18" s="40"/>
+      <c r="J18" s="39"/>
     </row>
     <row r="19" spans="1:10">
       <c r="A19">
@@ -21230,10 +21234,10 @@
       <c r="E19" t="s">
         <v>6247</v>
       </c>
-      <c r="G19" s="48"/>
-      <c r="H19" s="48"/>
-      <c r="I19" s="42"/>
-      <c r="J19" s="40"/>
+      <c r="G19" s="47"/>
+      <c r="H19" s="47"/>
+      <c r="I19" s="41"/>
+      <c r="J19" s="39"/>
     </row>
     <row r="20" spans="1:10">
       <c r="A20">
@@ -21251,10 +21255,10 @@
       <c r="E20" t="s">
         <v>6247</v>
       </c>
-      <c r="G20" s="48"/>
-      <c r="H20" s="48"/>
-      <c r="I20" s="42"/>
-      <c r="J20" s="40"/>
+      <c r="G20" s="47"/>
+      <c r="H20" s="47"/>
+      <c r="I20" s="41"/>
+      <c r="J20" s="39"/>
     </row>
     <row r="21" spans="1:10">
       <c r="A21">
@@ -21272,10 +21276,10 @@
       <c r="E21" t="s">
         <v>6247</v>
       </c>
-      <c r="G21" s="48"/>
-      <c r="H21" s="48"/>
-      <c r="I21" s="42"/>
-      <c r="J21" s="40"/>
+      <c r="G21" s="47"/>
+      <c r="H21" s="47"/>
+      <c r="I21" s="41"/>
+      <c r="J21" s="39"/>
     </row>
     <row r="22" spans="1:10">
       <c r="A22">
@@ -21293,10 +21297,10 @@
       <c r="E22" t="s">
         <v>6247</v>
       </c>
-      <c r="G22" s="48"/>
-      <c r="H22" s="48"/>
-      <c r="I22" s="42"/>
-      <c r="J22" s="40"/>
+      <c r="G22" s="47"/>
+      <c r="H22" s="47"/>
+      <c r="I22" s="41"/>
+      <c r="J22" s="39"/>
     </row>
     <row r="23" spans="1:10">
       <c r="A23">
@@ -21314,10 +21318,10 @@
       <c r="E23" t="s">
         <v>6247</v>
       </c>
-      <c r="G23" s="48"/>
-      <c r="H23" s="48"/>
-      <c r="I23" s="42"/>
-      <c r="J23" s="40"/>
+      <c r="G23" s="47"/>
+      <c r="H23" s="47"/>
+      <c r="I23" s="41"/>
+      <c r="J23" s="39"/>
     </row>
     <row r="24" spans="1:10">
       <c r="A24">
@@ -21335,10 +21339,10 @@
       <c r="E24" t="s">
         <v>6247</v>
       </c>
-      <c r="G24" s="48"/>
-      <c r="H24" s="48"/>
-      <c r="I24" s="42"/>
-      <c r="J24" s="40"/>
+      <c r="G24" s="47"/>
+      <c r="H24" s="47"/>
+      <c r="I24" s="41"/>
+      <c r="J24" s="39"/>
     </row>
     <row r="25" spans="1:10">
       <c r="A25">
@@ -21356,10 +21360,10 @@
       <c r="E25" t="s">
         <v>6247</v>
       </c>
-      <c r="G25" s="48"/>
-      <c r="H25" s="48"/>
-      <c r="I25" s="42"/>
-      <c r="J25" s="40"/>
+      <c r="G25" s="47"/>
+      <c r="H25" s="47"/>
+      <c r="I25" s="41"/>
+      <c r="J25" s="39"/>
     </row>
     <row r="26" spans="1:10">
       <c r="A26">
@@ -21377,10 +21381,10 @@
       <c r="E26" t="s">
         <v>6247</v>
       </c>
-      <c r="G26" s="48"/>
-      <c r="H26" s="48"/>
-      <c r="I26" s="42"/>
-      <c r="J26" s="40"/>
+      <c r="G26" s="47"/>
+      <c r="H26" s="47"/>
+      <c r="I26" s="41"/>
+      <c r="J26" s="39"/>
     </row>
     <row r="27" spans="1:10">
       <c r="A27">
@@ -21398,17 +21402,17 @@
       <c r="E27" t="s">
         <v>6247</v>
       </c>
-      <c r="G27" s="48" t="s">
+      <c r="G27" s="47" t="s">
         <v>6249</v>
       </c>
-      <c r="H27" s="41" t="e" cm="1" vm="5">
+      <c r="H27" s="40" t="e" cm="1" vm="5">
         <f t="array" ref="H27">_xlfn._xlws.PY(4,0)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="I27" s="42" t="s">
+      <c r="I27" s="41" t="s">
         <v>6248</v>
       </c>
-      <c r="J27" s="43"/>
+      <c r="J27" s="42"/>
     </row>
     <row r="28" spans="1:10">
       <c r="A28">
@@ -21426,10 +21430,10 @@
       <c r="E28" t="s">
         <v>6247</v>
       </c>
-      <c r="G28" s="48"/>
-      <c r="H28" s="41"/>
-      <c r="I28" s="42"/>
-      <c r="J28" s="44"/>
+      <c r="G28" s="47"/>
+      <c r="H28" s="40"/>
+      <c r="I28" s="41"/>
+      <c r="J28" s="43"/>
     </row>
     <row r="29" spans="1:10">
       <c r="A29">
@@ -21447,10 +21451,10 @@
       <c r="E29" t="s">
         <v>6247</v>
       </c>
-      <c r="G29" s="48"/>
-      <c r="H29" s="41"/>
-      <c r="I29" s="42"/>
-      <c r="J29" s="44"/>
+      <c r="G29" s="47"/>
+      <c r="H29" s="40"/>
+      <c r="I29" s="41"/>
+      <c r="J29" s="43"/>
     </row>
     <row r="30" spans="1:10">
       <c r="A30">
@@ -21468,10 +21472,10 @@
       <c r="E30" t="s">
         <v>6247</v>
       </c>
-      <c r="G30" s="48"/>
-      <c r="H30" s="41"/>
-      <c r="I30" s="42"/>
-      <c r="J30" s="44"/>
+      <c r="G30" s="47"/>
+      <c r="H30" s="40"/>
+      <c r="I30" s="41"/>
+      <c r="J30" s="43"/>
     </row>
     <row r="31" spans="1:10">
       <c r="A31">
@@ -21489,10 +21493,10 @@
       <c r="E31" t="s">
         <v>6247</v>
       </c>
-      <c r="G31" s="48"/>
-      <c r="H31" s="41"/>
-      <c r="I31" s="42"/>
-      <c r="J31" s="44"/>
+      <c r="G31" s="47"/>
+      <c r="H31" s="40"/>
+      <c r="I31" s="41"/>
+      <c r="J31" s="43"/>
     </row>
     <row r="32" spans="1:10">
       <c r="A32">
@@ -21510,10 +21514,10 @@
       <c r="E32" t="s">
         <v>6247</v>
       </c>
-      <c r="G32" s="48"/>
-      <c r="H32" s="41"/>
-      <c r="I32" s="42"/>
-      <c r="J32" s="44"/>
+      <c r="G32" s="47"/>
+      <c r="H32" s="40"/>
+      <c r="I32" s="41"/>
+      <c r="J32" s="43"/>
     </row>
     <row r="33" spans="1:10">
       <c r="A33">
@@ -21531,10 +21535,10 @@
       <c r="E33" t="s">
         <v>6247</v>
       </c>
-      <c r="G33" s="48"/>
-      <c r="H33" s="41"/>
-      <c r="I33" s="42"/>
-      <c r="J33" s="44"/>
+      <c r="G33" s="47"/>
+      <c r="H33" s="40"/>
+      <c r="I33" s="41"/>
+      <c r="J33" s="43"/>
     </row>
     <row r="34" spans="1:10">
       <c r="A34">
@@ -21552,10 +21556,10 @@
       <c r="E34" t="s">
         <v>6247</v>
       </c>
-      <c r="G34" s="48"/>
-      <c r="H34" s="41"/>
-      <c r="I34" s="42"/>
-      <c r="J34" s="44"/>
+      <c r="G34" s="47"/>
+      <c r="H34" s="40"/>
+      <c r="I34" s="41"/>
+      <c r="J34" s="43"/>
     </row>
     <row r="35" spans="1:10">
       <c r="A35">
@@ -21573,10 +21577,10 @@
       <c r="E35" t="s">
         <v>6247</v>
       </c>
-      <c r="G35" s="48"/>
-      <c r="H35" s="41"/>
-      <c r="I35" s="42"/>
-      <c r="J35" s="44"/>
+      <c r="G35" s="47"/>
+      <c r="H35" s="40"/>
+      <c r="I35" s="41"/>
+      <c r="J35" s="43"/>
     </row>
     <row r="36" spans="1:10">
       <c r="A36">
@@ -21594,10 +21598,10 @@
       <c r="E36" t="s">
         <v>6247</v>
       </c>
-      <c r="G36" s="48"/>
-      <c r="H36" s="41"/>
-      <c r="I36" s="42"/>
-      <c r="J36" s="44"/>
+      <c r="G36" s="47"/>
+      <c r="H36" s="40"/>
+      <c r="I36" s="41"/>
+      <c r="J36" s="43"/>
     </row>
     <row r="37" spans="1:10">
       <c r="A37">
@@ -21615,10 +21619,10 @@
       <c r="E37" t="s">
         <v>6247</v>
       </c>
-      <c r="G37" s="48"/>
-      <c r="H37" s="41"/>
-      <c r="I37" s="42"/>
-      <c r="J37" s="44"/>
+      <c r="G37" s="47"/>
+      <c r="H37" s="40"/>
+      <c r="I37" s="41"/>
+      <c r="J37" s="43"/>
     </row>
     <row r="38" spans="1:10">
       <c r="A38">
@@ -21636,10 +21640,10 @@
       <c r="E38" t="s">
         <v>6247</v>
       </c>
-      <c r="G38" s="48"/>
-      <c r="H38" s="41"/>
-      <c r="I38" s="42"/>
-      <c r="J38" s="44"/>
+      <c r="G38" s="47"/>
+      <c r="H38" s="40"/>
+      <c r="I38" s="41"/>
+      <c r="J38" s="43"/>
     </row>
     <row r="39" spans="1:10">
       <c r="A39">
@@ -21657,10 +21661,10 @@
       <c r="E39" t="s">
         <v>6247</v>
       </c>
-      <c r="G39" s="48"/>
-      <c r="H39" s="41"/>
-      <c r="I39" s="42"/>
-      <c r="J39" s="44"/>
+      <c r="G39" s="47"/>
+      <c r="H39" s="40"/>
+      <c r="I39" s="41"/>
+      <c r="J39" s="43"/>
     </row>
     <row r="40" spans="1:10">
       <c r="A40">
@@ -21678,10 +21682,10 @@
       <c r="E40" t="s">
         <v>6247</v>
       </c>
-      <c r="G40" s="48"/>
-      <c r="H40" s="41"/>
-      <c r="I40" s="42"/>
-      <c r="J40" s="45"/>
+      <c r="G40" s="47"/>
+      <c r="H40" s="40"/>
+      <c r="I40" s="41"/>
+      <c r="J40" s="44"/>
     </row>
     <row r="41" spans="1:10">
       <c r="A41">
@@ -23622,13 +23626,13 @@
       </c>
     </row>
     <row r="155" spans="1:5">
-      <c r="A155" s="50" t="s">
+      <c r="A155" s="49" t="s">
         <v>6244</v>
       </c>
-      <c r="B155" s="50"/>
-      <c r="C155" s="50"/>
-      <c r="D155" s="50"/>
-      <c r="E155" s="50"/>
+      <c r="B155" s="49"/>
+      <c r="C155" s="49"/>
+      <c r="D155" s="49"/>
+      <c r="E155" s="49"/>
     </row>
   </sheetData>
   <mergeCells count="23">
@@ -23677,15 +23681,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="23.25">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="48" t="s">
         <v>6269</v>
       </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="49"/>
-      <c r="F1" s="49"/>
-      <c r="G1" s="49"/>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
     </row>
     <row r="3" spans="1:10" ht="23.25">
       <c r="A3" s="15" t="s">
@@ -23693,10 +23697,10 @@
       </c>
       <c r="B3" s="14"/>
       <c r="C3" s="10"/>
-      <c r="G3" s="51" t="s">
+      <c r="G3" s="50" t="s">
         <v>6267</v>
       </c>
-      <c r="H3" s="51"/>
+      <c r="H3" s="50"/>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
@@ -23743,17 +23747,17 @@
       <c r="E5" t="s">
         <v>6247</v>
       </c>
-      <c r="G5" s="48" t="s">
+      <c r="G5" s="47" t="s">
         <v>6257</v>
       </c>
-      <c r="H5" s="41" t="e" cm="1" vm="1">
+      <c r="H5" s="40" t="e" cm="1" vm="1">
         <f t="array" ref="H5">_xlfn._xlws.PY(0,1,IrisDataSet[#All])</f>
         <v>#VALUE!</v>
       </c>
-      <c r="I5" s="42" t="s">
+      <c r="I5" s="41" t="s">
         <v>6256</v>
       </c>
-      <c r="J5" s="40"/>
+      <c r="J5" s="39"/>
     </row>
     <row r="6" spans="1:10">
       <c r="A6">
@@ -23771,10 +23775,10 @@
       <c r="E6" t="s">
         <v>6247</v>
       </c>
-      <c r="G6" s="48"/>
-      <c r="H6" s="41"/>
-      <c r="I6" s="42"/>
-      <c r="J6" s="40"/>
+      <c r="G6" s="47"/>
+      <c r="H6" s="40"/>
+      <c r="I6" s="41"/>
+      <c r="J6" s="39"/>
     </row>
     <row r="7" spans="1:10">
       <c r="A7">
@@ -23792,10 +23796,10 @@
       <c r="E7" t="s">
         <v>6247</v>
       </c>
-      <c r="G7" s="48"/>
-      <c r="H7" s="41"/>
-      <c r="I7" s="42"/>
-      <c r="J7" s="40"/>
+      <c r="G7" s="47"/>
+      <c r="H7" s="40"/>
+      <c r="I7" s="41"/>
+      <c r="J7" s="39"/>
     </row>
     <row r="8" spans="1:10">
       <c r="A8">
@@ -23813,10 +23817,10 @@
       <c r="E8" t="s">
         <v>6247</v>
       </c>
-      <c r="G8" s="48"/>
-      <c r="H8" s="41"/>
-      <c r="I8" s="42"/>
-      <c r="J8" s="40"/>
+      <c r="G8" s="47"/>
+      <c r="H8" s="40"/>
+      <c r="I8" s="41"/>
+      <c r="J8" s="39"/>
     </row>
     <row r="9" spans="1:10">
       <c r="A9">
@@ -23834,17 +23838,17 @@
       <c r="E9" t="s">
         <v>6247</v>
       </c>
-      <c r="G9" s="47" t="s">
+      <c r="G9" s="46" t="s">
         <v>6255</v>
       </c>
-      <c r="H9" s="41" t="e" cm="1" vm="2">
+      <c r="H9" s="40" t="e" cm="1" vm="2">
         <f t="array" ref="H9">_xlfn._xlws.PY(1,1)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="I9" s="42" t="s">
+      <c r="I9" s="41" t="s">
         <v>6254</v>
       </c>
-      <c r="J9" s="40"/>
+      <c r="J9" s="39"/>
     </row>
     <row r="10" spans="1:10">
       <c r="A10">
@@ -23862,10 +23866,10 @@
       <c r="E10" t="s">
         <v>6247</v>
       </c>
-      <c r="G10" s="48"/>
-      <c r="H10" s="41"/>
-      <c r="I10" s="42"/>
-      <c r="J10" s="40"/>
+      <c r="G10" s="47"/>
+      <c r="H10" s="40"/>
+      <c r="I10" s="41"/>
+      <c r="J10" s="39"/>
     </row>
     <row r="11" spans="1:10">
       <c r="A11">
@@ -23883,10 +23887,10 @@
       <c r="E11" t="s">
         <v>6247</v>
       </c>
-      <c r="G11" s="48"/>
-      <c r="H11" s="41"/>
-      <c r="I11" s="42"/>
-      <c r="J11" s="40"/>
+      <c r="G11" s="47"/>
+      <c r="H11" s="40"/>
+      <c r="I11" s="41"/>
+      <c r="J11" s="39"/>
     </row>
     <row r="12" spans="1:10">
       <c r="A12">
@@ -23904,10 +23908,10 @@
       <c r="E12" t="s">
         <v>6247</v>
       </c>
-      <c r="G12" s="48"/>
-      <c r="H12" s="41"/>
-      <c r="I12" s="42"/>
-      <c r="J12" s="40"/>
+      <c r="G12" s="47"/>
+      <c r="H12" s="40"/>
+      <c r="I12" s="41"/>
+      <c r="J12" s="39"/>
     </row>
     <row r="13" spans="1:10">
       <c r="A13">
@@ -23925,17 +23929,17 @@
       <c r="E13" t="s">
         <v>6247</v>
       </c>
-      <c r="G13" s="47" t="s">
+      <c r="G13" s="46" t="s">
         <v>6253</v>
       </c>
-      <c r="H13" s="41" t="e" cm="1" vm="3">
+      <c r="H13" s="40" t="e" cm="1" vm="3">
         <f t="array" ref="H13">_xlfn._xlws.PY(2,1)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="I13" s="42" t="s">
+      <c r="I13" s="41" t="s">
         <v>6252</v>
       </c>
-      <c r="J13" s="46"/>
+      <c r="J13" s="45"/>
     </row>
     <row r="14" spans="1:10">
       <c r="A14">
@@ -23953,10 +23957,10 @@
       <c r="E14" t="s">
         <v>6247</v>
       </c>
-      <c r="G14" s="48"/>
-      <c r="H14" s="41"/>
-      <c r="I14" s="42"/>
-      <c r="J14" s="46"/>
+      <c r="G14" s="47"/>
+      <c r="H14" s="40"/>
+      <c r="I14" s="41"/>
+      <c r="J14" s="45"/>
     </row>
     <row r="15" spans="1:10">
       <c r="A15">
@@ -23974,10 +23978,10 @@
       <c r="E15" t="s">
         <v>6247</v>
       </c>
-      <c r="G15" s="48"/>
-      <c r="H15" s="41"/>
-      <c r="I15" s="42"/>
-      <c r="J15" s="46"/>
+      <c r="G15" s="47"/>
+      <c r="H15" s="40"/>
+      <c r="I15" s="41"/>
+      <c r="J15" s="45"/>
     </row>
     <row r="16" spans="1:10">
       <c r="A16">
@@ -23995,10 +23999,10 @@
       <c r="E16" t="s">
         <v>6247</v>
       </c>
-      <c r="G16" s="48"/>
-      <c r="H16" s="41"/>
-      <c r="I16" s="42"/>
-      <c r="J16" s="46"/>
+      <c r="G16" s="47"/>
+      <c r="H16" s="40"/>
+      <c r="I16" s="41"/>
+      <c r="J16" s="45"/>
     </row>
     <row r="17" spans="1:10">
       <c r="A17">
@@ -24016,10 +24020,10 @@
       <c r="E17" t="s">
         <v>6247</v>
       </c>
-      <c r="G17" s="48"/>
-      <c r="H17" s="41"/>
-      <c r="I17" s="42"/>
-      <c r="J17" s="46"/>
+      <c r="G17" s="47"/>
+      <c r="H17" s="40"/>
+      <c r="I17" s="41"/>
+      <c r="J17" s="45"/>
     </row>
     <row r="18" spans="1:10">
       <c r="A18">
@@ -24037,17 +24041,17 @@
       <c r="E18" t="s">
         <v>6247</v>
       </c>
-      <c r="G18" s="47" t="s">
+      <c r="G18" s="46" t="s">
         <v>6251</v>
       </c>
-      <c r="H18" s="48" t="e" cm="1" vm="4">
+      <c r="H18" s="47" t="e" cm="1" vm="4">
         <f t="array" ref="H18">_xlfn._xlws.PY(3,0)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="I18" s="42" t="s">
+      <c r="I18" s="41" t="s">
         <v>6250</v>
       </c>
-      <c r="J18" s="40"/>
+      <c r="J18" s="39"/>
     </row>
     <row r="19" spans="1:10">
       <c r="A19">
@@ -24065,10 +24069,10 @@
       <c r="E19" t="s">
         <v>6247</v>
       </c>
-      <c r="G19" s="48"/>
-      <c r="H19" s="48"/>
-      <c r="I19" s="42"/>
-      <c r="J19" s="40"/>
+      <c r="G19" s="47"/>
+      <c r="H19" s="47"/>
+      <c r="I19" s="41"/>
+      <c r="J19" s="39"/>
     </row>
     <row r="20" spans="1:10">
       <c r="A20">
@@ -24086,10 +24090,10 @@
       <c r="E20" t="s">
         <v>6247</v>
       </c>
-      <c r="G20" s="48"/>
-      <c r="H20" s="48"/>
-      <c r="I20" s="42"/>
-      <c r="J20" s="40"/>
+      <c r="G20" s="47"/>
+      <c r="H20" s="47"/>
+      <c r="I20" s="41"/>
+      <c r="J20" s="39"/>
     </row>
     <row r="21" spans="1:10">
       <c r="A21">
@@ -24107,10 +24111,10 @@
       <c r="E21" t="s">
         <v>6247</v>
       </c>
-      <c r="G21" s="48"/>
-      <c r="H21" s="48"/>
-      <c r="I21" s="42"/>
-      <c r="J21" s="40"/>
+      <c r="G21" s="47"/>
+      <c r="H21" s="47"/>
+      <c r="I21" s="41"/>
+      <c r="J21" s="39"/>
     </row>
     <row r="22" spans="1:10">
       <c r="A22">
@@ -24128,10 +24132,10 @@
       <c r="E22" t="s">
         <v>6247</v>
       </c>
-      <c r="G22" s="48"/>
-      <c r="H22" s="48"/>
-      <c r="I22" s="42"/>
-      <c r="J22" s="40"/>
+      <c r="G22" s="47"/>
+      <c r="H22" s="47"/>
+      <c r="I22" s="41"/>
+      <c r="J22" s="39"/>
     </row>
     <row r="23" spans="1:10">
       <c r="A23">
@@ -24149,10 +24153,10 @@
       <c r="E23" t="s">
         <v>6247</v>
       </c>
-      <c r="G23" s="48"/>
-      <c r="H23" s="48"/>
-      <c r="I23" s="42"/>
-      <c r="J23" s="40"/>
+      <c r="G23" s="47"/>
+      <c r="H23" s="47"/>
+      <c r="I23" s="41"/>
+      <c r="J23" s="39"/>
     </row>
     <row r="24" spans="1:10">
       <c r="A24">
@@ -24170,10 +24174,10 @@
       <c r="E24" t="s">
         <v>6247</v>
       </c>
-      <c r="G24" s="48"/>
-      <c r="H24" s="48"/>
-      <c r="I24" s="42"/>
-      <c r="J24" s="40"/>
+      <c r="G24" s="47"/>
+      <c r="H24" s="47"/>
+      <c r="I24" s="41"/>
+      <c r="J24" s="39"/>
     </row>
     <row r="25" spans="1:10">
       <c r="A25">
@@ -24191,10 +24195,10 @@
       <c r="E25" t="s">
         <v>6247</v>
       </c>
-      <c r="G25" s="48"/>
-      <c r="H25" s="48"/>
-      <c r="I25" s="42"/>
-      <c r="J25" s="40"/>
+      <c r="G25" s="47"/>
+      <c r="H25" s="47"/>
+      <c r="I25" s="41"/>
+      <c r="J25" s="39"/>
     </row>
     <row r="26" spans="1:10">
       <c r="A26">
@@ -24212,10 +24216,10 @@
       <c r="E26" t="s">
         <v>6247</v>
       </c>
-      <c r="G26" s="48"/>
-      <c r="H26" s="48"/>
-      <c r="I26" s="42"/>
-      <c r="J26" s="40"/>
+      <c r="G26" s="47"/>
+      <c r="H26" s="47"/>
+      <c r="I26" s="41"/>
+      <c r="J26" s="39"/>
     </row>
     <row r="27" spans="1:10">
       <c r="A27">
@@ -24233,17 +24237,17 @@
       <c r="E27" t="s">
         <v>6247</v>
       </c>
-      <c r="G27" s="48" t="s">
+      <c r="G27" s="47" t="s">
         <v>6249</v>
       </c>
-      <c r="H27" s="41" t="e" cm="1" vm="5">
+      <c r="H27" s="40" t="e" cm="1" vm="5">
         <f t="array" ref="H27">_xlfn._xlws.PY(4,0)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="I27" s="42" t="s">
+      <c r="I27" s="41" t="s">
         <v>6248</v>
       </c>
-      <c r="J27" s="43"/>
+      <c r="J27" s="42"/>
     </row>
     <row r="28" spans="1:10">
       <c r="A28">
@@ -24261,10 +24265,10 @@
       <c r="E28" t="s">
         <v>6247</v>
       </c>
-      <c r="G28" s="48"/>
-      <c r="H28" s="41"/>
-      <c r="I28" s="42"/>
-      <c r="J28" s="44"/>
+      <c r="G28" s="47"/>
+      <c r="H28" s="40"/>
+      <c r="I28" s="41"/>
+      <c r="J28" s="43"/>
     </row>
     <row r="29" spans="1:10">
       <c r="A29">
@@ -24282,10 +24286,10 @@
       <c r="E29" t="s">
         <v>6247</v>
       </c>
-      <c r="G29" s="48"/>
-      <c r="H29" s="41"/>
-      <c r="I29" s="42"/>
-      <c r="J29" s="44"/>
+      <c r="G29" s="47"/>
+      <c r="H29" s="40"/>
+      <c r="I29" s="41"/>
+      <c r="J29" s="43"/>
     </row>
     <row r="30" spans="1:10">
       <c r="A30">
@@ -24303,10 +24307,10 @@
       <c r="E30" t="s">
         <v>6247</v>
       </c>
-      <c r="G30" s="48"/>
-      <c r="H30" s="41"/>
-      <c r="I30" s="42"/>
-      <c r="J30" s="44"/>
+      <c r="G30" s="47"/>
+      <c r="H30" s="40"/>
+      <c r="I30" s="41"/>
+      <c r="J30" s="43"/>
     </row>
     <row r="31" spans="1:10">
       <c r="A31">
@@ -24324,10 +24328,10 @@
       <c r="E31" t="s">
         <v>6247</v>
       </c>
-      <c r="G31" s="48"/>
-      <c r="H31" s="41"/>
-      <c r="I31" s="42"/>
-      <c r="J31" s="44"/>
+      <c r="G31" s="47"/>
+      <c r="H31" s="40"/>
+      <c r="I31" s="41"/>
+      <c r="J31" s="43"/>
     </row>
     <row r="32" spans="1:10">
       <c r="A32">
@@ -24345,10 +24349,10 @@
       <c r="E32" t="s">
         <v>6247</v>
       </c>
-      <c r="G32" s="48"/>
-      <c r="H32" s="41"/>
-      <c r="I32" s="42"/>
-      <c r="J32" s="44"/>
+      <c r="G32" s="47"/>
+      <c r="H32" s="40"/>
+      <c r="I32" s="41"/>
+      <c r="J32" s="43"/>
     </row>
     <row r="33" spans="1:10">
       <c r="A33">
@@ -24366,10 +24370,10 @@
       <c r="E33" t="s">
         <v>6247</v>
       </c>
-      <c r="G33" s="48"/>
-      <c r="H33" s="41"/>
-      <c r="I33" s="42"/>
-      <c r="J33" s="44"/>
+      <c r="G33" s="47"/>
+      <c r="H33" s="40"/>
+      <c r="I33" s="41"/>
+      <c r="J33" s="43"/>
     </row>
     <row r="34" spans="1:10">
       <c r="A34">
@@ -24387,10 +24391,10 @@
       <c r="E34" t="s">
         <v>6247</v>
       </c>
-      <c r="G34" s="48"/>
-      <c r="H34" s="41"/>
-      <c r="I34" s="42"/>
-      <c r="J34" s="44"/>
+      <c r="G34" s="47"/>
+      <c r="H34" s="40"/>
+      <c r="I34" s="41"/>
+      <c r="J34" s="43"/>
     </row>
     <row r="35" spans="1:10">
       <c r="A35">
@@ -24408,10 +24412,10 @@
       <c r="E35" t="s">
         <v>6247</v>
       </c>
-      <c r="G35" s="48"/>
-      <c r="H35" s="41"/>
-      <c r="I35" s="42"/>
-      <c r="J35" s="44"/>
+      <c r="G35" s="47"/>
+      <c r="H35" s="40"/>
+      <c r="I35" s="41"/>
+      <c r="J35" s="43"/>
     </row>
     <row r="36" spans="1:10">
       <c r="A36">
@@ -24429,10 +24433,10 @@
       <c r="E36" t="s">
         <v>6247</v>
       </c>
-      <c r="G36" s="48"/>
-      <c r="H36" s="41"/>
-      <c r="I36" s="42"/>
-      <c r="J36" s="44"/>
+      <c r="G36" s="47"/>
+      <c r="H36" s="40"/>
+      <c r="I36" s="41"/>
+      <c r="J36" s="43"/>
     </row>
     <row r="37" spans="1:10">
       <c r="A37">
@@ -24450,10 +24454,10 @@
       <c r="E37" t="s">
         <v>6247</v>
       </c>
-      <c r="G37" s="48"/>
-      <c r="H37" s="41"/>
-      <c r="I37" s="42"/>
-      <c r="J37" s="44"/>
+      <c r="G37" s="47"/>
+      <c r="H37" s="40"/>
+      <c r="I37" s="41"/>
+      <c r="J37" s="43"/>
     </row>
     <row r="38" spans="1:10">
       <c r="A38">
@@ -24471,10 +24475,10 @@
       <c r="E38" t="s">
         <v>6247</v>
       </c>
-      <c r="G38" s="48"/>
-      <c r="H38" s="41"/>
-      <c r="I38" s="42"/>
-      <c r="J38" s="44"/>
+      <c r="G38" s="47"/>
+      <c r="H38" s="40"/>
+      <c r="I38" s="41"/>
+      <c r="J38" s="43"/>
     </row>
     <row r="39" spans="1:10">
       <c r="A39">
@@ -24492,10 +24496,10 @@
       <c r="E39" t="s">
         <v>6247</v>
       </c>
-      <c r="G39" s="48"/>
-      <c r="H39" s="41"/>
-      <c r="I39" s="42"/>
-      <c r="J39" s="44"/>
+      <c r="G39" s="47"/>
+      <c r="H39" s="40"/>
+      <c r="I39" s="41"/>
+      <c r="J39" s="43"/>
     </row>
     <row r="40" spans="1:10">
       <c r="A40">
@@ -24513,10 +24517,10 @@
       <c r="E40" t="s">
         <v>6247</v>
       </c>
-      <c r="G40" s="48"/>
-      <c r="H40" s="41"/>
-      <c r="I40" s="42"/>
-      <c r="J40" s="45"/>
+      <c r="G40" s="47"/>
+      <c r="H40" s="40"/>
+      <c r="I40" s="41"/>
+      <c r="J40" s="44"/>
     </row>
     <row r="41" spans="1:10">
       <c r="A41">
@@ -26457,13 +26461,13 @@
       </c>
     </row>
     <row r="155" spans="1:5">
-      <c r="A155" s="50" t="s">
+      <c r="A155" s="49" t="s">
         <v>6244</v>
       </c>
-      <c r="B155" s="50"/>
-      <c r="C155" s="50"/>
-      <c r="D155" s="50"/>
-      <c r="E155" s="50"/>
+      <c r="B155" s="49"/>
+      <c r="C155" s="49"/>
+      <c r="D155" s="49"/>
+      <c r="E155" s="49"/>
     </row>
   </sheetData>
   <mergeCells count="23">
@@ -26578,17 +26582,17 @@
       <c r="D8" s="4"/>
     </row>
     <row r="9" spans="1:9" s="2" customFormat="1" ht="51" customHeight="1">
-      <c r="A9" s="52" t="s">
+      <c r="A9" s="51" t="s">
         <v>3263</v>
       </c>
-      <c r="B9" s="52"/>
-      <c r="C9" s="52"/>
-      <c r="D9" s="52"/>
-      <c r="E9" s="52"/>
-      <c r="F9" s="52"/>
-      <c r="G9" s="52"/>
-      <c r="H9" s="52"/>
-      <c r="I9" s="52"/>
+      <c r="B9" s="51"/>
+      <c r="C9" s="51"/>
+      <c r="D9" s="51"/>
+      <c r="E9" s="51"/>
+      <c r="F9" s="51"/>
+      <c r="G9" s="51"/>
+      <c r="H9" s="51"/>
+      <c r="I9" s="51"/>
     </row>
     <row r="10" spans="1:9" s="5" customFormat="1" ht="60">
       <c r="A10" s="8" t="s">
@@ -58600,64 +58604,64 @@
       </c>
     </row>
     <row r="1186" spans="1:11" s="2" customFormat="1">
-      <c r="A1186" s="53" t="s">
+      <c r="A1186" s="52" t="s">
         <v>6221</v>
       </c>
-      <c r="B1186" s="53"/>
-      <c r="C1186" s="53"/>
-      <c r="D1186" s="53"/>
-      <c r="E1186" s="53"/>
-      <c r="F1186" s="53"/>
-      <c r="G1186" s="53"/>
-      <c r="H1186" s="53"/>
-      <c r="I1186" s="53"/>
-      <c r="J1186" s="53"/>
-      <c r="K1186" s="53"/>
+      <c r="B1186" s="52"/>
+      <c r="C1186" s="52"/>
+      <c r="D1186" s="52"/>
+      <c r="E1186" s="52"/>
+      <c r="F1186" s="52"/>
+      <c r="G1186" s="52"/>
+      <c r="H1186" s="52"/>
+      <c r="I1186" s="52"/>
+      <c r="J1186" s="52"/>
+      <c r="K1186" s="52"/>
     </row>
     <row r="1187" spans="1:11" s="2" customFormat="1">
-      <c r="A1187" s="54" t="s">
+      <c r="A1187" s="53" t="s">
         <v>6218</v>
       </c>
-      <c r="B1187" s="54"/>
-      <c r="C1187" s="54"/>
-      <c r="D1187" s="54"/>
-      <c r="E1187" s="54"/>
-      <c r="F1187" s="54"/>
-      <c r="G1187" s="54"/>
-      <c r="H1187" s="54"/>
-      <c r="I1187" s="54"/>
-      <c r="J1187" s="54"/>
-      <c r="K1187" s="54"/>
+      <c r="B1187" s="53"/>
+      <c r="C1187" s="53"/>
+      <c r="D1187" s="53"/>
+      <c r="E1187" s="53"/>
+      <c r="F1187" s="53"/>
+      <c r="G1187" s="53"/>
+      <c r="H1187" s="53"/>
+      <c r="I1187" s="53"/>
+      <c r="J1187" s="53"/>
+      <c r="K1187" s="53"/>
     </row>
     <row r="1188" spans="1:11" s="2" customFormat="1">
-      <c r="A1188" s="54" t="s">
+      <c r="A1188" s="53" t="s">
         <v>6219</v>
       </c>
-      <c r="B1188" s="54"/>
-      <c r="C1188" s="54"/>
-      <c r="D1188" s="54"/>
-      <c r="E1188" s="54"/>
-      <c r="F1188" s="54"/>
-      <c r="G1188" s="54"/>
-      <c r="H1188" s="54"/>
-      <c r="I1188" s="54"/>
-      <c r="J1188" s="54"/>
-      <c r="K1188" s="54"/>
+      <c r="B1188" s="53"/>
+      <c r="C1188" s="53"/>
+      <c r="D1188" s="53"/>
+      <c r="E1188" s="53"/>
+      <c r="F1188" s="53"/>
+      <c r="G1188" s="53"/>
+      <c r="H1188" s="53"/>
+      <c r="I1188" s="53"/>
+      <c r="J1188" s="53"/>
+      <c r="K1188" s="53"/>
     </row>
     <row r="1189" spans="1:11" s="2" customFormat="1">
-      <c r="A1189" s="54" t="s">
+      <c r="A1189" s="53" t="s">
         <v>6220</v>
       </c>
-      <c r="B1189" s="54"/>
-      <c r="C1189" s="54"/>
-      <c r="D1189" s="54"/>
-      <c r="E1189" s="54"/>
-      <c r="F1189" s="54"/>
-      <c r="G1189" s="54"/>
-      <c r="H1189" s="54"/>
-      <c r="I1189" s="54"/>
-      <c r="J1189" s="54"/>
-      <c r="K1189" s="54"/>
+      <c r="B1189" s="53"/>
+      <c r="C1189" s="53"/>
+      <c r="D1189" s="53"/>
+      <c r="E1189" s="53"/>
+      <c r="F1189" s="53"/>
+      <c r="G1189" s="53"/>
+      <c r="H1189" s="53"/>
+      <c r="I1189" s="53"/>
+      <c r="J1189" s="53"/>
+      <c r="K1189" s="53"/>
     </row>
   </sheetData>
   <autoFilter ref="A10:I1184" xr:uid="{49C85161-1380-4812-A0F9-57BB38A11634}">
@@ -58714,25 +58718,25 @@
       </c>
       <c r="D1" s="59"/>
       <c r="E1" s="59"/>
-      <c r="F1" s="55" t="s">
+      <c r="F1" s="54" t="s">
         <v>6232</v>
       </c>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
+      <c r="G1" s="54"/>
+      <c r="H1" s="54"/>
       <c r="I1" s="19"/>
       <c r="J1" s="19"/>
       <c r="K1" s="19"/>
       <c r="L1" s="19"/>
-      <c r="M1" s="55" t="s">
+      <c r="M1" s="54" t="s">
         <v>6285</v>
       </c>
-      <c r="N1" s="55"/>
-      <c r="O1" s="55"/>
-      <c r="P1" s="55" t="s">
+      <c r="N1" s="54"/>
+      <c r="O1" s="54"/>
+      <c r="P1" s="54" t="s">
         <v>6235</v>
       </c>
-      <c r="Q1" s="55"/>
-      <c r="R1" s="55"/>
+      <c r="Q1" s="54"/>
+      <c r="R1" s="54"/>
     </row>
     <row r="2" spans="1:25" ht="15" customHeight="1">
       <c r="A2" s="58"/>
@@ -58819,10 +58823,10 @@
       <c r="S3" s="9"/>
     </row>
     <row r="4" spans="1:25" ht="16.5" thickTop="1" thickBot="1">
-      <c r="A4" s="39" t="s">
+      <c r="A4" s="55" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="56" t="s">
         <v>1176</v>
       </c>
       <c r="C4" t="s">
@@ -58875,12 +58879,8 @@
       </c>
     </row>
     <row r="5" spans="1:25" ht="16.5" thickTop="1" thickBot="1">
-      <c r="A5" s="39" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="23" t="s">
-        <v>1176</v>
-      </c>
+      <c r="A5" s="55"/>
+      <c r="B5" s="56"/>
       <c r="C5" t="s">
         <v>6239</v>
       </c>
@@ -58929,12 +58929,8 @@
       </c>
     </row>
     <row r="6" spans="1:25" ht="15.75" thickTop="1">
-      <c r="A6" s="39" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="23" t="s">
-        <v>1176</v>
-      </c>
+      <c r="A6" s="55"/>
+      <c r="B6" s="56"/>
       <c r="F6" s="56"/>
       <c r="G6" t="s">
         <v>6277</v>
@@ -58959,8 +58955,10 @@
       <c r="G7" s="10"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="11">
     <mergeCell ref="P1:R1"/>
+    <mergeCell ref="A4:A6"/>
+    <mergeCell ref="B4:B6"/>
     <mergeCell ref="G2:I2"/>
     <mergeCell ref="F4:F6"/>
     <mergeCell ref="A1:A2"/>

</xml_diff>